<commit_message>
changes to make it work
</commit_message>
<xml_diff>
--- a/Investment_Portfolio_Tracker.xlsx
+++ b/Investment_Portfolio_Tracker.xlsx
@@ -689,7 +689,7 @@
         <v>263.83</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>263.83</v>
+        <v>278.2250061035156</v>
       </c>
       <c r="F2" s="2">
         <f>C2*D2</f>
@@ -726,7 +726,7 @@
         <v>255.87</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>255.87</v>
+        <v>300.4500122070312</v>
       </c>
       <c r="F3" s="2">
         <f>C3*D3</f>
@@ -763,7 +763,7 @@
         <v>248.2</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>248.2</v>
+        <v>263.4400024414062</v>
       </c>
       <c r="F4" s="2">
         <f>C4*D4</f>
@@ -800,7 +800,7 @@
         <v>59.46</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>59.46</v>
+        <v>55.85010147094727</v>
       </c>
       <c r="F5" s="2">
         <f>C5*D5</f>
@@ -837,7 +837,7 @@
         <v>43.39</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>43.39</v>
+        <v>42.47499847412109</v>
       </c>
       <c r="F6" s="2">
         <f>C6*D6</f>
@@ -874,7 +874,7 @@
         <v>175.84</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>175.84</v>
+        <v>194.6750030517578</v>
       </c>
       <c r="F7" s="2">
         <f>C7*D7</f>
@@ -911,7 +911,7 @@
         <v>326.38</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>326.38</v>
+        <v>424.1099853515625</v>
       </c>
       <c r="F8" s="2">
         <f>C8*D8</f>
@@ -948,7 +948,7 @@
         <v>95.95</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>95.95</v>
+        <v>123.7649993896484</v>
       </c>
       <c r="F9" s="2">
         <f>C9*D9</f>
@@ -985,7 +985,7 @@
         <v>304.68</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>304.68</v>
+        <v>297.760009765625</v>
       </c>
       <c r="F10" s="2">
         <f>C10*D10</f>
@@ -1022,7 +1022,7 @@
         <v>153.54</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>153.54</v>
+        <v>732.25</v>
       </c>
       <c r="F11" s="2">
         <f>C11*D11</f>
@@ -1059,7 +1059,7 @@
         <v>27.75</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>27.75</v>
+        <v>27.03499984741211</v>
       </c>
       <c r="F12" s="2">
         <f>C12*D12</f>
@@ -1096,7 +1096,7 @@
         <v>3.7</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>3.7</v>
+        <v>5.054999828338623</v>
       </c>
       <c r="F13" s="2">
         <f>C13*D13</f>
@@ -1133,7 +1133,7 @@
         <v>45.88</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45.88</v>
+        <v>49.49499893188477</v>
       </c>
       <c r="F14" s="2">
         <f>C14*D14</f>
@@ -1170,7 +1170,7 @@
         <v>43.81</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>43.81</v>
+        <v>70.51999664306641</v>
       </c>
       <c r="F15" s="2">
         <f>C15*D15</f>
@@ -1207,7 +1207,7 @@
         <v>126.56</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>126.56</v>
+        <v>227.5500946044922</v>
       </c>
       <c r="F16" s="2">
         <f>C16*D16</f>
@@ -1244,7 +1244,7 @@
         <v>66.98999999999999</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>66.98999999999999</v>
+        <v>131.2599945068359</v>
       </c>
       <c r="F17" s="2">
         <f>C17*D17</f>
@@ -1281,7 +1281,7 @@
         <v>14.27</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>14.27</v>
+        <v>24.98999977111816</v>
       </c>
       <c r="F18" s="2">
         <f>C18*D18</f>
@@ -1318,7 +1318,7 @@
         <v>16.49</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>16.49</v>
+        <v>24.22500038146973</v>
       </c>
       <c r="F19" s="2">
         <f>C19*D19</f>
@@ -1814,28 +1814,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Portfolio Value: $1,616.01</t>
+          <t>Portfolio Value: $2,279.06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total Gain/Loss: $0.00</t>
+          <t>Total Gain/Loss: $663.05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Return %: 0.00%</t>
+          <t>Return %: 41.03%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Updated: 2026-05-15 19:07:41</t>
+          <t>Updated: 2026-05-15 19:19:54</t>
         </is>
       </c>
     </row>
@@ -1849,21 +1849,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Current Annual Return: 3780.00%</t>
+          <t>Current Annual Return: 27.35%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Current Risk (Volatility): 1093.16%</t>
+          <t>Current Risk (Volatility): 14.58%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Current Sharpe Ratio: 3.46</t>
+          <t>Current Sharpe Ratio: 1.88</t>
         </is>
       </c>
     </row>
@@ -1877,28 +1877,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Optimal Annual Return: 3780.00%</t>
+          <t>Optimal Annual Return: 86.58%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Optimal Risk (Volatility): 836.90%</t>
+          <t>Optimal Risk (Volatility): 18.88%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Optimal Sharpe Ratio: 4.52</t>
+          <t>Optimal Sharpe Ratio: 4.58</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Improvement in Sharpe: 30.6%</t>
+          <t>Improvement in Sharpe: 144.4%</t>
         </is>
       </c>
     </row>

</xml_diff>